<commit_message>
Update Physics For Computer Engineers resource file
</commit_message>
<xml_diff>
--- a/resources/Marks/2026/even/Physics For Computer Engineers.xlsx
+++ b/resources/Marks/2026/even/Physics For Computer Engineers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gusindia01-my.sharepoint.com/personal/nitesh_kumar_ddn_upes_ac_in/Documents/UPES/2026/Jan-May-2026/Physics for Computer Engineers B77 B78/Marks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2763" documentId="11_3FC952BF37FB7C428065D6D94F732ED04C5A5A3E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BC75CE4-3557-450F-9B3E-68E37A62BB12}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD4C6525-A239-4D5B-99DC-22605A8E80DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="553" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -782,7 +782,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -894,9 +894,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1138,7 +1135,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{121EC4BE-2A29-484F-96A3-3D5637F91420}" name="Table2" displayName="Table2" ref="A4:O65" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11">
-  <autoFilter ref="A4:O65" xr:uid="{121EC4BE-2A29-484F-96A3-3D5637F91420}"/>
+  <autoFilter ref="A4:O65" xr:uid="{121EC4BE-2A29-484F-96A3-3D5637F91420}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="78"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{C53A1133-970E-4861-9E6E-0807D65557FC}" name="Name" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{4B602A80-1925-4A20-94AA-A2291B2C30B5}" name="Student ID" dataDxfId="9"/>
@@ -1500,55 +1503,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
+      <c r="A1" s="43" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
       <c r="T1" s="24"/>
     </row>
     <row r="2" spans="1:22" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="43" t="s">
         <v>168</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
-      <c r="P2" s="44"/>
-      <c r="Q2" s="44"/>
-      <c r="R2" s="44"/>
-      <c r="S2" s="44"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
       <c r="T2" s="25"/>
     </row>
     <row r="3" spans="1:22" s="22" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="40" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="37" t="s">
@@ -1584,7 +1587,7 @@
       <c r="L3" s="37" t="s">
         <v>165</v>
       </c>
-      <c r="M3" s="42" t="s">
+      <c r="M3" s="41" t="s">
         <v>166</v>
       </c>
       <c r="N3" s="37" t="s">
@@ -1605,7 +1608,7 @@
       <c r="S3" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="U3" s="43" t="s">
+      <c r="U3" s="42" t="s">
         <v>13</v>
       </c>
       <c r="V3" s="23" t="s">
@@ -1767,7 +1770,7 @@
         <f t="shared" ref="J6:J63" si="0">SUM(D6:I6)</f>
         <v>41</v>
       </c>
-      <c r="K6" s="40"/>
+      <c r="K6" s="29"/>
       <c r="L6" s="29">
         <f t="shared" ref="L6:L63" si="1">SUM(J6:K6)/2</f>
         <v>20.5</v>
@@ -1833,7 +1836,7 @@
         <f t="shared" si="0"/>
         <v>29.2</v>
       </c>
-      <c r="K7" s="40"/>
+      <c r="K7" s="29"/>
       <c r="L7" s="29">
         <f t="shared" si="1"/>
         <v>14.6</v>
@@ -1899,7 +1902,7 @@
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="K8" s="40"/>
+      <c r="K8" s="29"/>
       <c r="L8" s="29">
         <f t="shared" si="1"/>
         <v>20.5</v>
@@ -1965,7 +1968,7 @@
         <f t="shared" si="0"/>
         <v>43.2</v>
       </c>
-      <c r="K9" s="40"/>
+      <c r="K9" s="29"/>
       <c r="L9" s="29">
         <f t="shared" si="1"/>
         <v>21.6</v>
@@ -2031,7 +2034,7 @@
         <f t="shared" si="0"/>
         <v>40.6</v>
       </c>
-      <c r="K10" s="40"/>
+      <c r="K10" s="29"/>
       <c r="L10" s="29">
         <f t="shared" si="1"/>
         <v>20.3</v>
@@ -2097,7 +2100,7 @@
         <f t="shared" si="0"/>
         <v>36.4</v>
       </c>
-      <c r="K11" s="40"/>
+      <c r="K11" s="29"/>
       <c r="L11" s="29">
         <f t="shared" si="1"/>
         <v>18.2</v>
@@ -2163,7 +2166,7 @@
         <f t="shared" si="0"/>
         <v>41.3</v>
       </c>
-      <c r="K12" s="40"/>
+      <c r="K12" s="29"/>
       <c r="L12" s="29">
         <f t="shared" si="1"/>
         <v>20.65</v>
@@ -2229,7 +2232,7 @@
         <f t="shared" si="0"/>
         <v>46.5</v>
       </c>
-      <c r="K13" s="40"/>
+      <c r="K13" s="29"/>
       <c r="L13" s="29">
         <f t="shared" si="1"/>
         <v>23.25</v>
@@ -2295,7 +2298,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K14" s="40"/>
+      <c r="K14" s="29"/>
       <c r="L14" s="29">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2361,7 +2364,7 @@
         <f t="shared" si="0"/>
         <v>33.200000000000003</v>
       </c>
-      <c r="K15" s="40"/>
+      <c r="K15" s="29"/>
       <c r="L15" s="29">
         <f t="shared" si="1"/>
         <v>16.600000000000001</v>
@@ -2427,7 +2430,7 @@
         <f t="shared" si="0"/>
         <v>38.9</v>
       </c>
-      <c r="K16" s="40"/>
+      <c r="K16" s="29"/>
       <c r="L16" s="29">
         <f t="shared" si="1"/>
         <v>19.45</v>
@@ -2493,7 +2496,7 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="K17" s="40"/>
+      <c r="K17" s="29"/>
       <c r="L17" s="29">
         <f t="shared" si="1"/>
         <v>16.5</v>
@@ -2559,7 +2562,7 @@
         <f t="shared" si="0"/>
         <v>33.200000000000003</v>
       </c>
-      <c r="K18" s="40"/>
+      <c r="K18" s="29"/>
       <c r="L18" s="29">
         <f t="shared" si="1"/>
         <v>16.600000000000001</v>
@@ -2625,7 +2628,7 @@
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="K19" s="40"/>
+      <c r="K19" s="29"/>
       <c r="L19" s="29">
         <f t="shared" si="1"/>
         <v>17.5</v>
@@ -2691,7 +2694,7 @@
         <f t="shared" si="0"/>
         <v>32.799999999999997</v>
       </c>
-      <c r="K20" s="40"/>
+      <c r="K20" s="29"/>
       <c r="L20" s="29">
         <f t="shared" si="1"/>
         <v>16.399999999999999</v>
@@ -2757,7 +2760,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K21" s="1"/>
+      <c r="K21" s="29"/>
       <c r="L21" s="29">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -2823,7 +2826,7 @@
         <f t="shared" si="0"/>
         <v>47.6</v>
       </c>
-      <c r="K22" s="1"/>
+      <c r="K22" s="29"/>
       <c r="L22" s="29">
         <f t="shared" si="1"/>
         <v>23.8</v>
@@ -2889,7 +2892,7 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="K23" s="1"/>
+      <c r="K23" s="29"/>
       <c r="L23" s="29">
         <f t="shared" si="1"/>
         <v>5.5</v>
@@ -2955,7 +2958,7 @@
         <f t="shared" si="0"/>
         <v>23.5</v>
       </c>
-      <c r="K24" s="1"/>
+      <c r="K24" s="29"/>
       <c r="L24" s="29">
         <f t="shared" si="1"/>
         <v>11.75</v>
@@ -3021,7 +3024,7 @@
         <f t="shared" si="0"/>
         <v>49.3</v>
       </c>
-      <c r="K25" s="1"/>
+      <c r="K25" s="29"/>
       <c r="L25" s="29">
         <f t="shared" si="1"/>
         <v>24.65</v>
@@ -3087,7 +3090,7 @@
         <f t="shared" si="0"/>
         <v>39.299999999999997</v>
       </c>
-      <c r="K26" s="1"/>
+      <c r="K26" s="29"/>
       <c r="L26" s="29">
         <f t="shared" si="1"/>
         <v>19.649999999999999</v>
@@ -3153,7 +3156,7 @@
         <f t="shared" si="0"/>
         <v>23.5</v>
       </c>
-      <c r="K27" s="1"/>
+      <c r="K27" s="29"/>
       <c r="L27" s="29">
         <f t="shared" si="1"/>
         <v>11.75</v>
@@ -3219,7 +3222,7 @@
         <f t="shared" si="0"/>
         <v>6.5</v>
       </c>
-      <c r="K28" s="1"/>
+      <c r="K28" s="29"/>
       <c r="L28" s="29">
         <f t="shared" si="1"/>
         <v>3.25</v>
@@ -3285,7 +3288,7 @@
         <f t="shared" si="0"/>
         <v>15.6</v>
       </c>
-      <c r="K29" s="1"/>
+      <c r="K29" s="29"/>
       <c r="L29" s="29">
         <f t="shared" si="1"/>
         <v>7.8</v>
@@ -3351,7 +3354,7 @@
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="K30" s="1"/>
+      <c r="K30" s="29"/>
       <c r="L30" s="29">
         <f t="shared" si="1"/>
         <v>17.5</v>
@@ -3417,7 +3420,7 @@
         <f t="shared" si="0"/>
         <v>40.4</v>
       </c>
-      <c r="K31" s="1"/>
+      <c r="K31" s="29"/>
       <c r="L31" s="29">
         <f t="shared" si="1"/>
         <v>20.2</v>
@@ -3483,7 +3486,7 @@
         <f t="shared" si="0"/>
         <v>45.6</v>
       </c>
-      <c r="K32" s="1"/>
+      <c r="K32" s="29"/>
       <c r="L32" s="29">
         <f t="shared" si="1"/>
         <v>22.8</v>
@@ -3549,7 +3552,7 @@
         <f t="shared" si="0"/>
         <v>49.5</v>
       </c>
-      <c r="K33" s="1"/>
+      <c r="K33" s="29"/>
       <c r="L33" s="29">
         <f t="shared" si="1"/>
         <v>24.75</v>
@@ -3615,7 +3618,7 @@
         <f t="shared" si="0"/>
         <v>38.6</v>
       </c>
-      <c r="K34" s="1"/>
+      <c r="K34" s="29"/>
       <c r="L34" s="29">
         <f t="shared" si="1"/>
         <v>19.3</v>
@@ -3626,11 +3629,11 @@
       </c>
       <c r="N34" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>7.6</v>
       </c>
       <c r="O34" s="29">
         <f>'Mid Sem'!O35</f>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="P34" s="29">
         <f>'End Sem'!N35</f>
@@ -3642,7 +3645,7 @@
       </c>
       <c r="R34" s="26">
         <f t="shared" si="5"/>
-        <v>9.65</v>
+        <v>17.25</v>
       </c>
       <c r="S34" s="36"/>
       <c r="U34" t="s">
@@ -3681,7 +3684,7 @@
         <f t="shared" si="0"/>
         <v>44.9</v>
       </c>
-      <c r="K35" s="1"/>
+      <c r="K35" s="29"/>
       <c r="L35" s="29">
         <f t="shared" si="1"/>
         <v>22.45</v>
@@ -3747,7 +3750,7 @@
         <f t="shared" si="0"/>
         <v>42.4</v>
       </c>
-      <c r="K36" s="1"/>
+      <c r="K36" s="29"/>
       <c r="L36" s="29">
         <f t="shared" si="1"/>
         <v>21.2</v>
@@ -3758,11 +3761,11 @@
       </c>
       <c r="N36" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="O36" s="29">
         <f>'Mid Sem'!O37</f>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="P36" s="29">
         <f>'End Sem'!N37</f>
@@ -3774,7 +3777,7 @@
       </c>
       <c r="R36" s="26">
         <f t="shared" si="5"/>
-        <v>10.6</v>
+        <v>16.8</v>
       </c>
       <c r="S36" s="36"/>
       <c r="U36" t="s">
@@ -3813,7 +3816,7 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="K37" s="1"/>
+      <c r="K37" s="29"/>
       <c r="L37" s="29">
         <f t="shared" si="1"/>
         <v>16.5</v>
@@ -3824,11 +3827,11 @@
       </c>
       <c r="N37" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>11.2</v>
       </c>
       <c r="O37" s="29">
         <f>'Mid Sem'!O38</f>
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="P37" s="29">
         <f>'End Sem'!N38</f>
@@ -3840,7 +3843,7 @@
       </c>
       <c r="R37" s="26">
         <f t="shared" si="5"/>
-        <v>8.25</v>
+        <v>19.45</v>
       </c>
       <c r="S37" s="36"/>
       <c r="U37" t="s">
@@ -3879,7 +3882,7 @@
         <f t="shared" si="0"/>
         <v>22.9</v>
       </c>
-      <c r="K38" s="1"/>
+      <c r="K38" s="29"/>
       <c r="L38" s="29">
         <f t="shared" si="1"/>
         <v>11.45</v>
@@ -3945,7 +3948,7 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="K39" s="1"/>
+      <c r="K39" s="29"/>
       <c r="L39" s="29">
         <f t="shared" si="1"/>
         <v>8</v>
@@ -4011,7 +4014,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="K40" s="1"/>
+      <c r="K40" s="29"/>
       <c r="L40" s="29">
         <f t="shared" si="1"/>
         <v>4</v>
@@ -4077,7 +4080,7 @@
         <f t="shared" si="0"/>
         <v>38.1</v>
       </c>
-      <c r="K41" s="1"/>
+      <c r="K41" s="29"/>
       <c r="L41" s="29">
         <f t="shared" si="1"/>
         <v>19.05</v>
@@ -4143,7 +4146,7 @@
         <f t="shared" si="0"/>
         <v>14.5</v>
       </c>
-      <c r="K42" s="1"/>
+      <c r="K42" s="29"/>
       <c r="L42" s="29">
         <f t="shared" si="1"/>
         <v>7.25</v>
@@ -4154,11 +4157,11 @@
       </c>
       <c r="N42" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="O42" s="29">
         <f>'Mid Sem'!O43</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P42" s="29">
         <f>'End Sem'!N43</f>
@@ -4170,7 +4173,7 @@
       </c>
       <c r="R42" s="26">
         <f t="shared" si="5"/>
-        <v>3.625</v>
+        <v>6.0250000000000004</v>
       </c>
       <c r="S42" s="1"/>
       <c r="U42" t="s">
@@ -4209,7 +4212,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K43" s="1"/>
+      <c r="K43" s="29"/>
       <c r="L43" s="29">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -4275,7 +4278,7 @@
         <f t="shared" si="0"/>
         <v>36.4</v>
       </c>
-      <c r="K44" s="1"/>
+      <c r="K44" s="29"/>
       <c r="L44" s="29">
         <f t="shared" si="1"/>
         <v>18.2</v>
@@ -4286,11 +4289,11 @@
       </c>
       <c r="N44" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="O44" s="29">
         <f>'Mid Sem'!O45</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P44" s="29">
         <f>'End Sem'!N45</f>
@@ -4302,7 +4305,7 @@
       </c>
       <c r="R44" s="26">
         <f t="shared" si="5"/>
-        <v>9.1</v>
+        <v>11.3</v>
       </c>
       <c r="S44" s="1"/>
       <c r="U44" t="s">
@@ -4341,7 +4344,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="K45" s="1"/>
+      <c r="K45" s="29"/>
       <c r="L45" s="29">
         <f t="shared" si="1"/>
         <v>7.5</v>
@@ -4407,7 +4410,7 @@
         <f t="shared" si="0"/>
         <v>36.299999999999997</v>
       </c>
-      <c r="K46" s="1"/>
+      <c r="K46" s="29"/>
       <c r="L46" s="29">
         <f t="shared" si="1"/>
         <v>18.149999999999999</v>
@@ -4418,11 +4421,11 @@
       </c>
       <c r="N46" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O46" s="29">
         <f>'Mid Sem'!O47</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P46" s="29">
         <f>'End Sem'!N47</f>
@@ -4434,7 +4437,7 @@
       </c>
       <c r="R46" s="26">
         <f t="shared" si="5"/>
-        <v>9.0749999999999993</v>
+        <v>11.074999999999999</v>
       </c>
       <c r="S46" s="1"/>
       <c r="U46" t="s">
@@ -4473,7 +4476,7 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="K47" s="1"/>
+      <c r="K47" s="29"/>
       <c r="L47" s="29">
         <f t="shared" si="1"/>
         <v>10.5</v>
@@ -4539,7 +4542,7 @@
         <f t="shared" si="0"/>
         <v>30.4</v>
       </c>
-      <c r="K48" s="1"/>
+      <c r="K48" s="29"/>
       <c r="L48" s="29">
         <f t="shared" si="1"/>
         <v>15.2</v>
@@ -4605,7 +4608,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K49" s="1"/>
+      <c r="K49" s="29"/>
       <c r="L49" s="29">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -4671,7 +4674,7 @@
         <f t="shared" si="0"/>
         <v>22.5</v>
       </c>
-      <c r="K50" s="1"/>
+      <c r="K50" s="29"/>
       <c r="L50" s="29">
         <f t="shared" si="1"/>
         <v>11.25</v>
@@ -4682,11 +4685,11 @@
       </c>
       <c r="N50" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="O50" s="29">
         <f>'Mid Sem'!O51</f>
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="P50" s="29">
         <f>'End Sem'!N51</f>
@@ -4698,7 +4701,7 @@
       </c>
       <c r="R50" s="26">
         <f t="shared" si="5"/>
-        <v>5.625</v>
+        <v>14.824999999999999</v>
       </c>
       <c r="S50" s="1"/>
       <c r="U50" t="s">
@@ -4737,7 +4740,7 @@
         <f t="shared" si="0"/>
         <v>45.9</v>
       </c>
-      <c r="K51" s="1"/>
+      <c r="K51" s="29"/>
       <c r="L51" s="29">
         <f t="shared" si="1"/>
         <v>22.95</v>
@@ -4748,11 +4751,11 @@
       </c>
       <c r="N51" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="O51" s="29">
         <f>'Mid Sem'!O52</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P51" s="29">
         <f>'End Sem'!N52</f>
@@ -4764,7 +4767,7 @@
       </c>
       <c r="R51" s="26">
         <f t="shared" si="5"/>
-        <v>11.475</v>
+        <v>11.674999999999999</v>
       </c>
       <c r="S51" s="1"/>
       <c r="U51" t="s">
@@ -4803,7 +4806,7 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="K52" s="1"/>
+      <c r="K52" s="29"/>
       <c r="L52" s="29">
         <f t="shared" si="1"/>
         <v>3.5</v>
@@ -4814,11 +4817,11 @@
       </c>
       <c r="N52" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="O52" s="29">
         <f>'Mid Sem'!O53</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P52" s="29">
         <f>'End Sem'!N53</f>
@@ -4830,7 +4833,7 @@
       </c>
       <c r="R52" s="26">
         <f t="shared" si="5"/>
-        <v>1.75</v>
+        <v>1.95</v>
       </c>
       <c r="S52" s="1"/>
       <c r="U52" t="s">
@@ -4880,11 +4883,11 @@
       </c>
       <c r="N53" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="O53" s="29">
         <f>'Mid Sem'!O54</f>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="P53" s="29">
         <f>'End Sem'!N54</f>
@@ -4896,7 +4899,7 @@
       </c>
       <c r="R53" s="26">
         <f t="shared" si="5"/>
-        <v>9.4749999999999996</v>
+        <v>12.875</v>
       </c>
       <c r="S53" s="1"/>
       <c r="U53" t="s">
@@ -4946,11 +4949,11 @@
       </c>
       <c r="N54" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="O54" s="29">
         <f>'Mid Sem'!O55</f>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="P54" s="29">
         <f>'End Sem'!N55</f>
@@ -4962,7 +4965,7 @@
       </c>
       <c r="R54" s="26">
         <f t="shared" si="5"/>
-        <v>11.275</v>
+        <v>14.675000000000001</v>
       </c>
       <c r="S54" s="1"/>
       <c r="U54" t="s">
@@ -5078,11 +5081,11 @@
       </c>
       <c r="N56" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="O56" s="29">
         <f>'Mid Sem'!O57</f>
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="P56" s="29">
         <f>'End Sem'!N57</f>
@@ -5094,7 +5097,7 @@
       </c>
       <c r="R56" s="26">
         <f t="shared" si="5"/>
-        <v>8.25</v>
+        <v>12.65</v>
       </c>
       <c r="S56" s="1"/>
       <c r="U56" t="s">
@@ -5144,11 +5147,11 @@
       </c>
       <c r="N57" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="O57" s="29">
         <f>'Mid Sem'!O58</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P57" s="29">
         <f>'End Sem'!N58</f>
@@ -5160,7 +5163,7 @@
       </c>
       <c r="R57" s="26">
         <f t="shared" si="5"/>
-        <v>6.75</v>
+        <v>8.5500000000000007</v>
       </c>
       <c r="S57" s="1"/>
       <c r="U57" t="s">
@@ -5210,11 +5213,11 @@
       </c>
       <c r="N58" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="O58" s="29">
         <f>'Mid Sem'!O59</f>
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="P58" s="29">
         <f>'End Sem'!N59</f>
@@ -5226,7 +5229,7 @@
       </c>
       <c r="R58" s="26">
         <f t="shared" si="5"/>
-        <v>11.45</v>
+        <v>27.849999999999998</v>
       </c>
       <c r="S58" s="1"/>
       <c r="U58" t="s">
@@ -5276,11 +5279,11 @@
       </c>
       <c r="N59" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="O59" s="29">
         <f>'Mid Sem'!O60</f>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="P59" s="29">
         <f>'End Sem'!N60</f>
@@ -5292,7 +5295,7 @@
       </c>
       <c r="R59" s="26">
         <f t="shared" si="5"/>
-        <v>10.375</v>
+        <v>16.574999999999999</v>
       </c>
       <c r="S59" s="1"/>
       <c r="U59" t="s">
@@ -5342,11 +5345,11 @@
       </c>
       <c r="N60" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>13.6</v>
       </c>
       <c r="O60" s="29">
         <f>'Mid Sem'!O61</f>
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="P60" s="29">
         <f>'End Sem'!N61</f>
@@ -5358,7 +5361,7 @@
       </c>
       <c r="R60" s="26">
         <f t="shared" si="5"/>
-        <v>10.175000000000001</v>
+        <v>23.774999999999999</v>
       </c>
       <c r="S60" s="1"/>
       <c r="U60" t="s">
@@ -5408,11 +5411,11 @@
       </c>
       <c r="N61" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O61" s="29">
         <f>'Mid Sem'!O62</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="P61" s="29">
         <f>'End Sem'!N62</f>
@@ -5424,7 +5427,7 @@
       </c>
       <c r="R61" s="26">
         <f t="shared" si="5"/>
-        <v>11.3</v>
+        <v>23.3</v>
       </c>
       <c r="S61" s="1"/>
       <c r="U61" t="s">
@@ -5474,11 +5477,11 @@
       </c>
       <c r="N62" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>12.6</v>
       </c>
       <c r="O62" s="29">
         <f>'Mid Sem'!O63</f>
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="P62" s="29">
         <f>'End Sem'!N63</f>
@@ -5490,7 +5493,7 @@
       </c>
       <c r="R62" s="26">
         <f t="shared" si="5"/>
-        <v>9.5</v>
+        <v>22.1</v>
       </c>
       <c r="S62" s="1"/>
       <c r="U62" t="s">
@@ -5540,11 +5543,11 @@
       </c>
       <c r="N63" s="29">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="O63" s="29">
         <f>'Mid Sem'!O64</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="P63" s="29">
         <f>'End Sem'!N64</f>
@@ -5556,7 +5559,7 @@
       </c>
       <c r="R63" s="26">
         <f t="shared" si="5"/>
-        <v>11.375</v>
+        <v>13.975</v>
       </c>
       <c r="S63" s="1"/>
       <c r="U63" t="s">
@@ -5750,11 +5753,11 @@
       </c>
       <c r="N67">
         <f>MEDIAN(N5:N63)</f>
-        <v>0.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="O67">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="P67">
         <f t="shared" si="8"/>
@@ -5766,7 +5769,7 @@
       </c>
       <c r="R67">
         <f t="shared" si="8"/>
-        <v>11.225</v>
+        <v>13.975</v>
       </c>
       <c r="S67" t="e">
         <f t="shared" si="8"/>
@@ -5835,7 +5838,7 @@
       </c>
       <c r="R68" cm="1">
         <f t="array" ref="R68">MEDIAN(_xlfn._xlws.FILTER(R5:R63, R5:R63&lt;&gt;0))</f>
-        <v>11.287500000000001</v>
+        <v>14.3375</v>
       </c>
     </row>
   </sheetData>
@@ -8407,45 +8410,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>162</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
     </row>
     <row r="2" spans="1:21" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="str">
+      <c r="A2" s="43" t="str">
         <f>Marksheet!A2</f>
         <v xml:space="preserve">Physics for Computer Engineers (PHYS 1036) </v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -12038,47 +12041,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
     </row>
     <row r="2" spans="1:22" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="str">
+      <c r="A2" s="43" t="str">
         <f>Marksheet!A2</f>
         <v xml:space="preserve">Physics for Computer Engineers (PHYS 1036) </v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -15358,45 +15361,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
     </row>
     <row r="2" spans="1:21" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="str">
+      <c r="A2" s="43" t="str">
         <f>Marksheet!A2</f>
         <v xml:space="preserve">Physics for Computer Engineers (PHYS 1036) </v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -15495,7 +15498,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
       <c r="B5" s="8" t="s">
         <v>15</v>
@@ -15548,7 +15551,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="str">
         <f>Marksheet!A5</f>
         <v>Aadya Dubey</v>
@@ -15607,7 +15610,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="str">
         <f>Marksheet!A6</f>
         <v>Aditya Vishwakarma</v>
@@ -15660,7 +15663,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="31" t="str">
         <f>Marksheet!A7</f>
         <v>Arjun</v>
@@ -15713,7 +15716,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="str">
         <f>Marksheet!A8</f>
         <v>Aryan Yadav</v>
@@ -15770,7 +15773,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="str">
         <f>Marksheet!A9</f>
         <v>Astik Patel</v>
@@ -15829,7 +15832,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="str">
         <f>Marksheet!A10</f>
         <v>Ayush Mohan</v>
@@ -15878,7 +15881,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="str">
         <f>Marksheet!A11</f>
         <v>Bhanu Purohit</v>
@@ -15937,7 +15940,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="str">
         <f>Marksheet!A12</f>
         <v>Biswabandya Mohanty</v>
@@ -15982,7 +15985,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="str">
         <f>Marksheet!A13</f>
         <v>Eashan Vashisht</v>
@@ -16041,7 +16044,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="31" t="str">
         <f>Marksheet!A14</f>
         <v>Hardik Joshi</v>
@@ -16082,7 +16085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="str">
         <f>Marksheet!A15</f>
         <v>Hrithvik Bhardwaj</v>
@@ -16125,7 +16128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="str">
         <f>Marksheet!A16</f>
         <v>Nitish Kumar</v>
@@ -16180,7 +16183,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="str">
         <f>Marksheet!A17</f>
         <v>Omkareshwar Chaubey</v>
@@ -16239,7 +16242,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="str">
         <f>Marksheet!A18</f>
         <v>Pavani Jain</v>
@@ -16298,7 +16301,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="31" t="str">
         <f>Marksheet!A19</f>
         <v>Prapti Uniyal</v>
@@ -16357,7 +16360,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="str">
         <f>Marksheet!A20</f>
         <v>Priyadarshi Prabhakar</v>
@@ -16410,7 +16413,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="str">
         <f>Marksheet!A21</f>
         <v>Radhe Patel</v>
@@ -16469,7 +16472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="str">
         <f>Marksheet!A22</f>
         <v>Rishika Purushotham</v>
@@ -16524,7 +16527,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="str">
         <f>Marksheet!A23</f>
         <v>Rishiv Kumar</v>
@@ -16573,7 +16576,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="str">
         <f>Marksheet!A24</f>
         <v>Sankalp Sunil Ronge</v>
@@ -16620,7 +16623,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="31" t="str">
         <f>Marksheet!A25</f>
         <v>Sartaj Singh</v>
@@ -16679,7 +16682,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="31" t="str">
         <f>Marksheet!A26</f>
         <v>Satakshi Gupta</v>
@@ -16732,7 +16735,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="31" t="str">
         <f>Marksheet!A27</f>
         <v>Shaswat Shantanu</v>
@@ -16781,7 +16784,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="31" t="str">
         <f>Marksheet!A28</f>
         <v>Siddhant Rai</v>
@@ -16830,7 +16833,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="31" t="str">
         <f>Marksheet!A29</f>
         <v>Sidhaant Singh Jyrwa</v>
@@ -16875,7 +16878,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="31" t="str">
         <f>Marksheet!A30</f>
         <v>Subrat Singh Jadaun</v>
@@ -16928,7 +16931,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="31" t="str">
         <f>Marksheet!A31</f>
         <v>Tushita Sharma</v>
@@ -16987,7 +16990,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="31" t="str">
         <f>Marksheet!A32</f>
         <v>Vaishnavi Kumari</v>
@@ -17038,7 +17041,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="31" t="str">
         <f>Marksheet!A33</f>
         <v>Vivek Chauhan</v>
@@ -17109,33 +17112,51 @@
       <c r="C35" s="12">
         <v>78</v>
       </c>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
+      <c r="D35" s="10">
+        <v>3</v>
+      </c>
+      <c r="E35" s="10">
+        <v>6</v>
+      </c>
+      <c r="F35" s="10">
+        <v>5</v>
+      </c>
+      <c r="G35" s="10">
+        <v>0</v>
+      </c>
+      <c r="H35" s="10">
+        <v>4</v>
+      </c>
+      <c r="I35" s="10">
+        <v>5</v>
+      </c>
+      <c r="J35" s="10">
+        <v>13</v>
+      </c>
+      <c r="K35" s="10">
+        <v>0</v>
+      </c>
+      <c r="L35" s="10">
+        <v>2</v>
+      </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
       <c r="O35" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="P35" s="9"/>
       <c r="S35" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>36.4</v>
       </c>
       <c r="T35" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="U35" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -17150,15 +17171,33 @@
       <c r="C36" s="12">
         <v>78</v>
       </c>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="10"/>
+      <c r="D36" s="10">
+        <v>0</v>
+      </c>
+      <c r="E36" s="10">
+        <v>0</v>
+      </c>
+      <c r="F36" s="10">
+        <v>0</v>
+      </c>
+      <c r="G36" s="10">
+        <v>0</v>
+      </c>
+      <c r="H36" s="10">
+        <v>0</v>
+      </c>
+      <c r="I36" s="10">
+        <v>0</v>
+      </c>
+      <c r="J36" s="10">
+        <v>0</v>
+      </c>
+      <c r="K36" s="10">
+        <v>0</v>
+      </c>
+      <c r="L36" s="10">
+        <v>0</v>
+      </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
       <c r="O36" s="14">
@@ -17191,25 +17230,43 @@
       <c r="C37" s="12">
         <v>78</v>
       </c>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
-      <c r="I37" s="10"/>
-      <c r="J37" s="10"/>
-      <c r="K37" s="10"/>
-      <c r="L37" s="10"/>
+      <c r="D37" s="10">
+        <v>6</v>
+      </c>
+      <c r="E37" s="10">
+        <v>4</v>
+      </c>
+      <c r="F37" s="10">
+        <v>5</v>
+      </c>
+      <c r="G37" s="10">
+        <v>0</v>
+      </c>
+      <c r="H37" s="10">
+        <v>0</v>
+      </c>
+      <c r="I37" s="10">
+        <v>13</v>
+      </c>
+      <c r="J37" s="10">
+        <v>3</v>
+      </c>
+      <c r="K37" s="10">
+        <v>0</v>
+      </c>
+      <c r="L37" s="10">
+        <v>0</v>
+      </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
       <c r="O37" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="P37" s="9"/>
       <c r="S37" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="T37" s="26">
         <f t="shared" si="2"/>
@@ -17217,7 +17274,7 @@
       </c>
       <c r="U37" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -17232,33 +17289,51 @@
       <c r="C38" s="12">
         <v>78</v>
       </c>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="10"/>
-      <c r="G38" s="10"/>
-      <c r="H38" s="10"/>
-      <c r="I38" s="10"/>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10"/>
-      <c r="L38" s="10"/>
+      <c r="D38" s="10">
+        <v>4</v>
+      </c>
+      <c r="E38" s="10">
+        <v>6</v>
+      </c>
+      <c r="F38" s="10">
+        <v>5</v>
+      </c>
+      <c r="G38" s="10">
+        <v>2</v>
+      </c>
+      <c r="H38" s="10">
+        <v>5</v>
+      </c>
+      <c r="I38" s="10">
+        <v>15</v>
+      </c>
+      <c r="J38" s="10">
+        <v>12</v>
+      </c>
+      <c r="K38" s="10">
+        <v>2</v>
+      </c>
+      <c r="L38" s="10">
+        <v>5</v>
+      </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>
       <c r="O38" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="P38" s="9"/>
       <c r="S38" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="T38" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="U38" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>56</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
@@ -17276,14 +17351,30 @@
       <c r="D39" s="10">
         <v>2</v>
       </c>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
-      <c r="I39" s="10"/>
-      <c r="J39" s="10"/>
-      <c r="K39" s="10"/>
-      <c r="L39" s="10"/>
+      <c r="E39" s="10">
+        <v>0</v>
+      </c>
+      <c r="F39" s="10">
+        <v>0</v>
+      </c>
+      <c r="G39" s="10">
+        <v>0</v>
+      </c>
+      <c r="H39" s="10">
+        <v>0</v>
+      </c>
+      <c r="I39" s="10">
+        <v>0</v>
+      </c>
+      <c r="J39" s="10">
+        <v>0</v>
+      </c>
+      <c r="K39" s="10">
+        <v>0</v>
+      </c>
+      <c r="L39" s="10">
+        <v>0</v>
+      </c>
       <c r="M39" s="10"/>
       <c r="N39" s="10"/>
       <c r="O39" s="14">
@@ -17455,8 +17546,12 @@
       <c r="J42" s="10">
         <v>3</v>
       </c>
-      <c r="K42" s="10"/>
-      <c r="L42" s="10"/>
+      <c r="K42" s="10">
+        <v>0</v>
+      </c>
+      <c r="L42" s="10">
+        <v>0</v>
+      </c>
       <c r="M42" s="10"/>
       <c r="N42" s="10"/>
       <c r="O42" s="14">
@@ -17489,25 +17584,43 @@
       <c r="C43" s="12">
         <v>78</v>
       </c>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
-      <c r="H43" s="10"/>
-      <c r="I43" s="10"/>
-      <c r="J43" s="10"/>
-      <c r="K43" s="10"/>
-      <c r="L43" s="10"/>
+      <c r="D43" s="10">
+        <v>6</v>
+      </c>
+      <c r="E43" s="10">
+        <v>4</v>
+      </c>
+      <c r="F43" s="10">
+        <v>0</v>
+      </c>
+      <c r="G43" s="10">
+        <v>0</v>
+      </c>
+      <c r="H43" s="10">
+        <v>0</v>
+      </c>
+      <c r="I43" s="10">
+        <v>2</v>
+      </c>
+      <c r="J43" s="10">
+        <v>0</v>
+      </c>
+      <c r="K43" s="10">
+        <v>0</v>
+      </c>
+      <c r="L43" s="10">
+        <v>0</v>
+      </c>
       <c r="M43" s="10"/>
       <c r="N43" s="10"/>
       <c r="O43" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P43" s="9"/>
       <c r="S43" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="T43" s="26">
         <f t="shared" si="2"/>
@@ -17515,7 +17628,7 @@
       </c>
       <c r="U43" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -17530,15 +17643,33 @@
       <c r="C44" s="12">
         <v>78</v>
       </c>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
+      <c r="D44" s="10">
+        <v>0</v>
+      </c>
+      <c r="E44" s="10">
+        <v>0</v>
+      </c>
+      <c r="F44" s="10">
+        <v>0</v>
+      </c>
+      <c r="G44" s="10">
+        <v>0</v>
+      </c>
+      <c r="H44" s="10">
+        <v>0</v>
+      </c>
+      <c r="I44" s="10">
+        <v>0</v>
+      </c>
+      <c r="J44" s="10">
+        <v>0</v>
+      </c>
+      <c r="K44" s="10">
+        <v>0</v>
+      </c>
+      <c r="L44" s="10">
+        <v>0</v>
+      </c>
       <c r="M44" s="10"/>
       <c r="N44" s="10"/>
       <c r="O44" s="14">
@@ -17571,25 +17702,43 @@
       <c r="C45" s="12">
         <v>78</v>
       </c>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="10"/>
-      <c r="H45" s="10"/>
-      <c r="I45" s="10"/>
-      <c r="J45" s="10"/>
-      <c r="K45" s="10"/>
-      <c r="L45" s="10"/>
+      <c r="D45" s="10">
+        <v>4</v>
+      </c>
+      <c r="E45" s="10">
+        <v>3</v>
+      </c>
+      <c r="F45" s="10">
+        <v>1</v>
+      </c>
+      <c r="G45" s="10">
+        <v>0</v>
+      </c>
+      <c r="H45" s="10">
+        <v>1</v>
+      </c>
+      <c r="I45" s="10">
+        <v>2</v>
+      </c>
+      <c r="J45" s="10">
+        <v>0</v>
+      </c>
+      <c r="K45" s="10">
+        <v>0</v>
+      </c>
+      <c r="L45" s="10">
+        <v>0</v>
+      </c>
       <c r="M45" s="10"/>
       <c r="N45" s="10"/>
       <c r="O45" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="P45" s="9"/>
       <c r="S45" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="T45" s="26">
         <f t="shared" si="2"/>
@@ -17597,7 +17746,7 @@
       </c>
       <c r="U45" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -17612,15 +17761,33 @@
       <c r="C46" s="12">
         <v>78</v>
       </c>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10"/>
-      <c r="I46" s="10"/>
-      <c r="J46" s="10"/>
-      <c r="K46" s="10"/>
-      <c r="L46" s="10"/>
+      <c r="D46" s="10">
+        <v>0</v>
+      </c>
+      <c r="E46" s="10">
+        <v>0</v>
+      </c>
+      <c r="F46" s="10">
+        <v>0</v>
+      </c>
+      <c r="G46" s="10">
+        <v>0</v>
+      </c>
+      <c r="H46" s="10">
+        <v>0</v>
+      </c>
+      <c r="I46" s="10">
+        <v>0</v>
+      </c>
+      <c r="J46" s="10">
+        <v>0</v>
+      </c>
+      <c r="K46" s="10">
+        <v>0</v>
+      </c>
+      <c r="L46" s="10">
+        <v>0</v>
+      </c>
       <c r="M46" s="10"/>
       <c r="N46" s="10"/>
       <c r="O46" s="14">
@@ -17653,33 +17820,51 @@
       <c r="C47" s="12">
         <v>78</v>
       </c>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
-      <c r="G47" s="10"/>
-      <c r="H47" s="10"/>
-      <c r="I47" s="10"/>
-      <c r="J47" s="10"/>
-      <c r="K47" s="10"/>
-      <c r="L47" s="10"/>
+      <c r="D47" s="10">
+        <v>4</v>
+      </c>
+      <c r="E47" s="10">
+        <v>2</v>
+      </c>
+      <c r="F47" s="10">
+        <v>0</v>
+      </c>
+      <c r="G47" s="10">
+        <v>2</v>
+      </c>
+      <c r="H47" s="10">
+        <v>1</v>
+      </c>
+      <c r="I47" s="10">
+        <v>0</v>
+      </c>
+      <c r="J47" s="10">
+        <v>1</v>
+      </c>
+      <c r="K47" s="10">
+        <v>0</v>
+      </c>
+      <c r="L47" s="10">
+        <v>0</v>
+      </c>
       <c r="M47" s="10"/>
       <c r="N47" s="10"/>
       <c r="O47" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P47" s="9"/>
       <c r="S47" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="T47" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U47" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
@@ -17700,13 +17885,27 @@
       <c r="E48" s="10">
         <v>4</v>
       </c>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
-      <c r="I48" s="10"/>
-      <c r="J48" s="10"/>
-      <c r="K48" s="10"/>
-      <c r="L48" s="10"/>
+      <c r="F48" s="10">
+        <v>0</v>
+      </c>
+      <c r="G48" s="10">
+        <v>0</v>
+      </c>
+      <c r="H48" s="10">
+        <v>0</v>
+      </c>
+      <c r="I48" s="10">
+        <v>0</v>
+      </c>
+      <c r="J48" s="10">
+        <v>0</v>
+      </c>
+      <c r="K48" s="10">
+        <v>0</v>
+      </c>
+      <c r="L48" s="10">
+        <v>0</v>
+      </c>
       <c r="M48" s="10"/>
       <c r="N48" s="10"/>
       <c r="O48" s="14">
@@ -17739,15 +17938,33 @@
       <c r="C49" s="12">
         <v>78</v>
       </c>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
-      <c r="F49" s="10"/>
-      <c r="G49" s="10"/>
-      <c r="H49" s="10"/>
-      <c r="I49" s="10"/>
-      <c r="J49" s="10"/>
-      <c r="K49" s="10"/>
-      <c r="L49" s="10"/>
+      <c r="D49" s="10">
+        <v>0</v>
+      </c>
+      <c r="E49" s="10">
+        <v>0</v>
+      </c>
+      <c r="F49" s="10">
+        <v>0</v>
+      </c>
+      <c r="G49" s="10">
+        <v>0</v>
+      </c>
+      <c r="H49" s="10">
+        <v>0</v>
+      </c>
+      <c r="I49" s="10">
+        <v>0</v>
+      </c>
+      <c r="J49" s="10">
+        <v>0</v>
+      </c>
+      <c r="K49" s="10">
+        <v>0</v>
+      </c>
+      <c r="L49" s="10">
+        <v>0</v>
+      </c>
       <c r="M49" s="10"/>
       <c r="N49" s="10"/>
       <c r="O49" s="14">
@@ -17780,15 +17997,33 @@
       <c r="C50" s="12">
         <v>78</v>
       </c>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="10"/>
-      <c r="H50" s="10"/>
-      <c r="I50" s="10"/>
-      <c r="J50" s="10"/>
-      <c r="K50" s="10"/>
-      <c r="L50" s="10"/>
+      <c r="D50" s="10">
+        <v>0</v>
+      </c>
+      <c r="E50" s="10">
+        <v>0</v>
+      </c>
+      <c r="F50" s="10">
+        <v>0</v>
+      </c>
+      <c r="G50" s="10">
+        <v>0</v>
+      </c>
+      <c r="H50" s="10">
+        <v>0</v>
+      </c>
+      <c r="I50" s="10">
+        <v>0</v>
+      </c>
+      <c r="J50" s="10">
+        <v>0</v>
+      </c>
+      <c r="K50" s="10">
+        <v>0</v>
+      </c>
+      <c r="L50" s="10">
+        <v>0</v>
+      </c>
       <c r="M50" s="10"/>
       <c r="N50" s="10"/>
       <c r="O50" s="14">
@@ -17821,33 +18056,51 @@
       <c r="C51" s="12">
         <v>78</v>
       </c>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="10"/>
-      <c r="G51" s="10"/>
-      <c r="H51" s="10"/>
-      <c r="I51" s="10"/>
-      <c r="J51" s="10"/>
-      <c r="K51" s="10"/>
-      <c r="L51" s="10"/>
+      <c r="D51" s="10">
+        <v>4</v>
+      </c>
+      <c r="E51" s="10">
+        <v>4</v>
+      </c>
+      <c r="F51" s="10">
+        <v>6</v>
+      </c>
+      <c r="G51" s="10">
+        <v>4</v>
+      </c>
+      <c r="H51" s="10">
+        <v>2</v>
+      </c>
+      <c r="I51" s="10">
+        <v>12</v>
+      </c>
+      <c r="J51" s="10">
+        <v>12</v>
+      </c>
+      <c r="K51" s="10">
+        <v>0</v>
+      </c>
+      <c r="L51" s="10">
+        <v>2</v>
+      </c>
       <c r="M51" s="10"/>
       <c r="N51" s="10"/>
       <c r="O51" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="P51" s="9"/>
       <c r="S51" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>40.4</v>
       </c>
       <c r="T51" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="U51" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -17862,25 +18115,43 @@
       <c r="C52" s="12">
         <v>78</v>
       </c>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
-      <c r="G52" s="10"/>
-      <c r="H52" s="10"/>
-      <c r="I52" s="10"/>
-      <c r="J52" s="10"/>
-      <c r="K52" s="10"/>
-      <c r="L52" s="10"/>
+      <c r="D52" s="10">
+        <v>1</v>
+      </c>
+      <c r="E52" s="10">
+        <v>0</v>
+      </c>
+      <c r="F52" s="10">
+        <v>0</v>
+      </c>
+      <c r="G52" s="10">
+        <v>0</v>
+      </c>
+      <c r="H52" s="10">
+        <v>0</v>
+      </c>
+      <c r="I52" s="10">
+        <v>0</v>
+      </c>
+      <c r="J52" s="10">
+        <v>0</v>
+      </c>
+      <c r="K52" s="10">
+        <v>0</v>
+      </c>
+      <c r="L52" s="10">
+        <v>0</v>
+      </c>
       <c r="M52" s="10"/>
       <c r="N52" s="10"/>
       <c r="O52" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P52" s="9"/>
       <c r="S52" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T52" s="26">
         <f t="shared" si="2"/>
@@ -17888,7 +18159,7 @@
       </c>
       <c r="U52" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -17903,25 +18174,43 @@
       <c r="C53" s="12">
         <v>78</v>
       </c>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="10"/>
-      <c r="G53" s="10"/>
-      <c r="H53" s="10"/>
-      <c r="I53" s="10"/>
-      <c r="J53" s="10"/>
-      <c r="K53" s="10"/>
-      <c r="L53" s="10"/>
+      <c r="D53" s="10">
+        <v>0</v>
+      </c>
+      <c r="E53" s="10">
+        <v>0</v>
+      </c>
+      <c r="F53" s="10">
+        <v>0</v>
+      </c>
+      <c r="G53" s="10">
+        <v>0</v>
+      </c>
+      <c r="H53" s="10">
+        <v>0</v>
+      </c>
+      <c r="I53" s="10">
+        <v>0</v>
+      </c>
+      <c r="J53" s="10">
+        <v>1</v>
+      </c>
+      <c r="K53" s="10">
+        <v>0</v>
+      </c>
+      <c r="L53" s="10">
+        <v>0</v>
+      </c>
       <c r="M53" s="10"/>
       <c r="N53" s="10"/>
       <c r="O53" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P53" s="9"/>
       <c r="S53" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T53" s="26">
         <f t="shared" si="2"/>
@@ -17929,7 +18218,7 @@
       </c>
       <c r="U53" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -17944,25 +18233,43 @@
       <c r="C54" s="12">
         <v>78</v>
       </c>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="10"/>
-      <c r="G54" s="10"/>
-      <c r="H54" s="10"/>
-      <c r="I54" s="10"/>
-      <c r="J54" s="10"/>
-      <c r="K54" s="10"/>
-      <c r="L54" s="10"/>
+      <c r="D54" s="10">
+        <v>6</v>
+      </c>
+      <c r="E54" s="10">
+        <v>5</v>
+      </c>
+      <c r="F54" s="10">
+        <v>0</v>
+      </c>
+      <c r="G54" s="10">
+        <v>0</v>
+      </c>
+      <c r="H54" s="10">
+        <v>0</v>
+      </c>
+      <c r="I54" s="10">
+        <v>6</v>
+      </c>
+      <c r="J54" s="10">
+        <v>0</v>
+      </c>
+      <c r="K54" s="10">
+        <v>0</v>
+      </c>
+      <c r="L54" s="10">
+        <v>0</v>
+      </c>
       <c r="M54" s="10"/>
       <c r="N54" s="10"/>
       <c r="O54" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="P54" s="9"/>
       <c r="S54" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="T54" s="26">
         <f t="shared" si="2"/>
@@ -17970,7 +18277,7 @@
       </c>
       <c r="U54" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
@@ -17985,33 +18292,51 @@
       <c r="C55" s="12">
         <v>78</v>
       </c>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="10"/>
-      <c r="H55" s="10"/>
-      <c r="I55" s="10"/>
-      <c r="J55" s="10"/>
-      <c r="K55" s="10"/>
-      <c r="L55" s="10"/>
+      <c r="D55" s="10">
+        <v>2</v>
+      </c>
+      <c r="E55" s="10">
+        <v>2</v>
+      </c>
+      <c r="F55" s="10">
+        <v>4</v>
+      </c>
+      <c r="G55" s="10">
+        <v>0</v>
+      </c>
+      <c r="H55" s="10">
+        <v>2</v>
+      </c>
+      <c r="I55" s="10">
+        <v>2</v>
+      </c>
+      <c r="J55" s="10">
+        <v>4</v>
+      </c>
+      <c r="K55" s="10">
+        <v>0</v>
+      </c>
+      <c r="L55" s="10">
+        <v>1</v>
+      </c>
       <c r="M55" s="10"/>
       <c r="N55" s="10"/>
       <c r="O55" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="P55" s="9"/>
       <c r="S55" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>16.2</v>
       </c>
       <c r="T55" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="U55" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -18026,15 +18351,33 @@
       <c r="C56" s="12">
         <v>78</v>
       </c>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="10"/>
-      <c r="G56" s="10"/>
-      <c r="H56" s="10"/>
-      <c r="I56" s="10"/>
-      <c r="J56" s="10"/>
-      <c r="K56" s="10"/>
-      <c r="L56" s="10"/>
+      <c r="D56" s="10">
+        <v>0</v>
+      </c>
+      <c r="E56" s="10">
+        <v>0</v>
+      </c>
+      <c r="F56" s="10">
+        <v>0</v>
+      </c>
+      <c r="G56" s="10">
+        <v>0</v>
+      </c>
+      <c r="H56" s="10">
+        <v>0</v>
+      </c>
+      <c r="I56" s="10">
+        <v>0</v>
+      </c>
+      <c r="J56" s="10">
+        <v>0</v>
+      </c>
+      <c r="K56" s="10">
+        <v>0</v>
+      </c>
+      <c r="L56" s="10">
+        <v>0</v>
+      </c>
       <c r="M56" s="10"/>
       <c r="N56" s="10"/>
       <c r="O56" s="14">
@@ -18067,33 +18410,51 @@
       <c r="C57" s="12">
         <v>78</v>
       </c>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="10"/>
-      <c r="G57" s="10"/>
-      <c r="H57" s="10"/>
-      <c r="I57" s="10"/>
-      <c r="J57" s="10"/>
-      <c r="K57" s="10"/>
-      <c r="L57" s="10"/>
+      <c r="D57" s="10">
+        <v>4</v>
+      </c>
+      <c r="E57" s="10">
+        <v>1</v>
+      </c>
+      <c r="F57" s="10">
+        <v>4</v>
+      </c>
+      <c r="G57" s="10">
+        <v>0</v>
+      </c>
+      <c r="H57" s="10">
+        <v>0</v>
+      </c>
+      <c r="I57" s="10">
+        <v>3</v>
+      </c>
+      <c r="J57" s="10">
+        <v>0</v>
+      </c>
+      <c r="K57" s="10">
+        <v>0</v>
+      </c>
+      <c r="L57" s="10">
+        <v>10</v>
+      </c>
       <c r="M57" s="10"/>
       <c r="N57" s="10"/>
       <c r="O57" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="P57" s="9"/>
       <c r="S57" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="T57" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="U57" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -18108,25 +18469,43 @@
       <c r="C58" s="12">
         <v>78</v>
       </c>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
-      <c r="H58" s="10"/>
-      <c r="I58" s="10"/>
-      <c r="J58" s="10"/>
-      <c r="K58" s="10"/>
-      <c r="L58" s="10"/>
+      <c r="D58" s="10">
+        <v>4</v>
+      </c>
+      <c r="E58" s="10">
+        <v>0</v>
+      </c>
+      <c r="F58" s="10">
+        <v>0</v>
+      </c>
+      <c r="G58" s="10">
+        <v>0</v>
+      </c>
+      <c r="H58" s="10">
+        <v>0</v>
+      </c>
+      <c r="I58" s="10">
+        <v>5</v>
+      </c>
+      <c r="J58" s="10">
+        <v>0</v>
+      </c>
+      <c r="K58" s="10">
+        <v>0</v>
+      </c>
+      <c r="L58" s="10">
+        <v>0</v>
+      </c>
       <c r="M58" s="10"/>
       <c r="N58" s="10"/>
       <c r="O58" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P58" s="9"/>
       <c r="S58" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="T58" s="26">
         <f t="shared" si="2"/>
@@ -18134,7 +18513,7 @@
       </c>
       <c r="U58" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -18149,33 +18528,51 @@
       <c r="C59" s="12">
         <v>78</v>
       </c>
-      <c r="D59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
-      <c r="G59" s="10"/>
-      <c r="H59" s="10"/>
-      <c r="I59" s="10"/>
-      <c r="J59" s="10"/>
-      <c r="K59" s="10"/>
-      <c r="L59" s="10"/>
+      <c r="D59" s="10">
+        <v>6</v>
+      </c>
+      <c r="E59" s="10">
+        <v>6</v>
+      </c>
+      <c r="F59" s="10">
+        <v>5</v>
+      </c>
+      <c r="G59" s="10">
+        <v>4</v>
+      </c>
+      <c r="H59" s="10">
+        <v>6</v>
+      </c>
+      <c r="I59" s="10">
+        <v>15</v>
+      </c>
+      <c r="J59" s="10">
+        <v>15</v>
+      </c>
+      <c r="K59" s="10">
+        <v>10</v>
+      </c>
+      <c r="L59" s="10">
+        <v>15</v>
+      </c>
       <c r="M59" s="10"/>
       <c r="N59" s="10"/>
       <c r="O59" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="P59" s="9"/>
       <c r="S59" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="T59" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="U59" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -18190,33 +18587,51 @@
       <c r="C60" s="12">
         <v>78</v>
       </c>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
-      <c r="H60" s="10"/>
-      <c r="I60" s="10"/>
-      <c r="J60" s="10"/>
-      <c r="K60" s="10"/>
-      <c r="L60" s="10"/>
+      <c r="D60" s="10">
+        <v>4</v>
+      </c>
+      <c r="E60" s="10">
+        <v>0</v>
+      </c>
+      <c r="F60" s="10">
+        <v>0</v>
+      </c>
+      <c r="G60" s="10">
+        <v>0</v>
+      </c>
+      <c r="H60" s="10">
+        <v>2</v>
+      </c>
+      <c r="I60" s="10">
+        <v>7</v>
+      </c>
+      <c r="J60" s="10">
+        <v>3</v>
+      </c>
+      <c r="K60" s="10">
+        <v>0</v>
+      </c>
+      <c r="L60" s="10">
+        <v>15</v>
+      </c>
       <c r="M60" s="10"/>
       <c r="N60" s="10"/>
       <c r="O60" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="P60" s="9"/>
       <c r="S60" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="T60" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="U60" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>31</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -18231,33 +18646,51 @@
       <c r="C61" s="12">
         <v>78</v>
       </c>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
-      <c r="H61" s="10"/>
-      <c r="I61" s="10"/>
-      <c r="J61" s="10"/>
-      <c r="K61" s="10"/>
-      <c r="L61" s="10"/>
+      <c r="D61" s="10">
+        <v>6</v>
+      </c>
+      <c r="E61" s="10">
+        <v>5.5</v>
+      </c>
+      <c r="F61" s="10">
+        <v>6</v>
+      </c>
+      <c r="G61" s="10">
+        <v>5.5</v>
+      </c>
+      <c r="H61" s="10">
+        <v>3</v>
+      </c>
+      <c r="I61" s="10">
+        <v>15</v>
+      </c>
+      <c r="J61" s="10">
+        <v>15</v>
+      </c>
+      <c r="K61" s="10">
+        <v>3</v>
+      </c>
+      <c r="L61" s="10">
+        <v>9</v>
+      </c>
       <c r="M61" s="10"/>
       <c r="N61" s="10"/>
       <c r="O61" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="P61" s="9"/>
       <c r="S61" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>52.3</v>
       </c>
       <c r="T61" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>15.7</v>
       </c>
       <c r="U61" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>68</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -18272,33 +18705,51 @@
       <c r="C62" s="12">
         <v>78</v>
       </c>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="10"/>
-      <c r="G62" s="10"/>
-      <c r="H62" s="10"/>
-      <c r="I62" s="10"/>
-      <c r="J62" s="10"/>
-      <c r="K62" s="10"/>
-      <c r="L62" s="10"/>
+      <c r="D62" s="10">
+        <v>6</v>
+      </c>
+      <c r="E62" s="10">
+        <v>6</v>
+      </c>
+      <c r="F62" s="10">
+        <v>6</v>
+      </c>
+      <c r="G62" s="10">
+        <v>4</v>
+      </c>
+      <c r="H62" s="10">
+        <v>4</v>
+      </c>
+      <c r="I62" s="10">
+        <v>14</v>
+      </c>
+      <c r="J62" s="10">
+        <v>5</v>
+      </c>
+      <c r="K62" s="10">
+        <v>5</v>
+      </c>
+      <c r="L62" s="10">
+        <v>10</v>
+      </c>
       <c r="M62" s="10"/>
       <c r="N62" s="10"/>
       <c r="O62" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="P62" s="9"/>
       <c r="S62" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="T62" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="U62" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -18313,33 +18764,51 @@
       <c r="C63" s="12">
         <v>78</v>
       </c>
-      <c r="D63" s="10"/>
-      <c r="E63" s="10"/>
-      <c r="F63" s="10"/>
-      <c r="G63" s="10"/>
-      <c r="H63" s="10"/>
-      <c r="I63" s="10"/>
-      <c r="J63" s="10"/>
-      <c r="K63" s="10"/>
-      <c r="L63" s="10"/>
+      <c r="D63" s="10">
+        <v>4</v>
+      </c>
+      <c r="E63" s="10">
+        <v>6</v>
+      </c>
+      <c r="F63" s="10">
+        <v>6</v>
+      </c>
+      <c r="G63" s="10">
+        <v>2</v>
+      </c>
+      <c r="H63" s="10">
+        <v>5</v>
+      </c>
+      <c r="I63" s="10">
+        <v>10</v>
+      </c>
+      <c r="J63" s="10">
+        <v>15</v>
+      </c>
+      <c r="K63" s="10">
+        <v>5</v>
+      </c>
+      <c r="L63" s="10">
+        <v>10</v>
+      </c>
       <c r="M63" s="10"/>
       <c r="N63" s="10"/>
       <c r="O63" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="P63" s="9"/>
       <c r="S63" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="T63" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="U63" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>63</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -18354,36 +18823,54 @@
       <c r="C64" s="12">
         <v>78</v>
       </c>
-      <c r="D64" s="10"/>
-      <c r="E64" s="10"/>
-      <c r="F64" s="10"/>
-      <c r="G64" s="10"/>
-      <c r="H64" s="10"/>
-      <c r="I64" s="10"/>
-      <c r="J64" s="10"/>
-      <c r="K64" s="10"/>
-      <c r="L64" s="10"/>
+      <c r="D64" s="10">
+        <v>1</v>
+      </c>
+      <c r="E64" s="10">
+        <v>2</v>
+      </c>
+      <c r="F64" s="10">
+        <v>3</v>
+      </c>
+      <c r="G64" s="10">
+        <v>0</v>
+      </c>
+      <c r="H64" s="10">
+        <v>0</v>
+      </c>
+      <c r="I64" s="10">
+        <v>2</v>
+      </c>
+      <c r="J64" s="10">
+        <v>0</v>
+      </c>
+      <c r="K64" s="10">
+        <v>0</v>
+      </c>
+      <c r="L64" s="10">
+        <v>5</v>
+      </c>
       <c r="M64" s="10"/>
       <c r="N64" s="10"/>
       <c r="O64" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="P64" s="9"/>
       <c r="S64" s="26">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="T64" s="26">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U64" s="26">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="65" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="31"/>
       <c r="C65" s="12"/>
       <c r="D65" s="10"/>
@@ -18443,43 +18930,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
     </row>
     <row r="2" spans="1:15" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="str">
+      <c r="A2" s="43" t="str">
         <f>Marksheet!A2</f>
         <v xml:space="preserve">Physics for Computer Engineers (PHYS 1036) </v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
@@ -19465,43 +19952,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
     </row>
     <row r="2" spans="1:15" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="str">
+      <c r="A2" s="43" t="str">
         <f>Marksheet!A2</f>
         <v xml:space="preserve">Physics for Computer Engineers (PHYS 1036) </v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -20452,43 +20939,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
     </row>
     <row r="2" spans="1:20" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="str">
+      <c r="A2" s="43" t="str">
         <f>Marksheet!A2</f>
         <v xml:space="preserve">Physics for Computer Engineers (PHYS 1036) </v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -23802,43 +24289,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
     </row>
     <row r="2" spans="1:15" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="str">
+      <c r="A2" s="43" t="str">
         <f>Marksheet!A2</f>
         <v xml:space="preserve">Physics for Computer Engineers (PHYS 1036) </v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -24788,43 +25275,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
     </row>
     <row r="2" spans="1:15" ht="24.75" x14ac:dyDescent="0.4">
-      <c r="A2" s="44" t="str">
+      <c r="A2" s="43" t="str">
         <f>Marksheet!A2</f>
         <v xml:space="preserve">Physics for Computer Engineers (PHYS 1036) </v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>

</xml_diff>

<commit_message>
Remove unused lab score calculations and related UI elements from marks portal
</commit_message>
<xml_diff>
--- a/resources/Marks/2026/even/Physics For Computer Engineers.xlsx
+++ b/resources/Marks/2026/even/Physics For Computer Engineers.xlsx
@@ -1336,7 +1336,7 @@
     <col min="7" max="7" style="22" width="14.290714285714287" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="22" width="14.290714285714287" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="22" width="14.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="70" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="70" width="16.719285714285714" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="22" width="11.862142857142858" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="70" width="11.862142857142858" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="70" width="11.147857142857141" customWidth="1" bestFit="1"/>
@@ -1550,9 +1550,7 @@
       <c r="J5" s="3">
         <f>SUM(D5:I5)</f>
       </c>
-      <c r="K5" s="21">
-        <v>2</v>
-      </c>
+      <c r="K5" s="21"/>
       <c r="L5" s="66">
         <f>SUM(J5:K5)/2</f>
       </c>

</xml_diff>